<commit_message>
fixed all comments on license and description, made vignettes mroe robust, fixed errors in the functions making them more accessable
</commit_message>
<xml_diff>
--- a/valuation_data.xlsx
+++ b/valuation_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/66e327b93913c047/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="128" documentId="8_{255DDA58-B8F0-4DA9-9842-F736A8E69B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24034AD3-DEBF-4B40-9DAD-1E1A046FB779}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="8_{255DDA58-B8F0-4DA9-9842-F736A8E69B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA85D4BF-1E49-42A3-B33D-E2DA855DA83D}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0E020BBE-65F7-4622-B4B9-D4D68F80CABC}"/>
+    <workbookView minimized="1" xWindow="4800" yWindow="3110" windowWidth="14400" windowHeight="8170" xr2:uid="{0E020BBE-65F7-4622-B4B9-D4D68F80CABC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="45">
   <si>
     <t>Company Name</t>
   </si>
@@ -174,18 +174,6 @@
   </si>
   <si>
     <t>Net Debt</t>
-  </si>
-  <si>
-    <t>P/E</t>
-  </si>
-  <si>
-    <t>EV/Revenue</t>
-  </si>
-  <si>
-    <t>EV/EBITDA</t>
-  </si>
-  <si>
-    <t>Net Income Margin</t>
   </si>
 </sst>
 </file>
@@ -280,6 +268,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -670,18 +662,10 @@
       <c r="N1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>48</v>
-      </c>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+      <c r="R1" s="5"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -730,22 +714,10 @@
         <f>J2/I2</f>
         <v>0.24152542372881355</v>
       </c>
-      <c r="O2" s="8">
-        <f>D2/L2</f>
-        <v>13.985507246376811</v>
-      </c>
-      <c r="P2" s="6">
-        <f>H2/I2</f>
-        <v>2.3728813559322033</v>
-      </c>
-      <c r="Q2" s="6">
-        <f>H2/J2</f>
-        <v>9.8245614035087723</v>
-      </c>
-      <c r="R2" s="7">
-        <f>K2/I2</f>
-        <v>0.1461864406779661</v>
-      </c>
+      <c r="O2" s="8"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="7"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -794,22 +766,10 @@
         <f t="shared" ref="N3:N16" si="3">J3/I3</f>
         <v>0.18474576271186441</v>
       </c>
-      <c r="O3" s="6">
-        <f t="shared" ref="O3:O16" si="4">D3/L3</f>
-        <v>12.6412213740458</v>
-      </c>
-      <c r="P3" s="6">
-        <f t="shared" ref="P3:P16" si="5">H3/I3</f>
-        <v>1.7317796610169491</v>
-      </c>
-      <c r="Q3" s="6">
-        <f t="shared" ref="Q3:Q16" si="6">H3/J3</f>
-        <v>9.373853211009175</v>
-      </c>
-      <c r="R3" s="7">
-        <f t="shared" ref="R3:R16" si="7">K3/I3</f>
-        <v>0.11101694915254237</v>
-      </c>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="7"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -858,22 +818,10 @@
         <f t="shared" si="3"/>
         <v>0.15466101694915255</v>
       </c>
-      <c r="O4" s="6">
-        <f t="shared" si="4"/>
-        <v>18.122448979591837</v>
-      </c>
-      <c r="P4" s="6">
-        <f t="shared" si="5"/>
-        <v>1.8334745762711864</v>
-      </c>
-      <c r="Q4" s="6">
-        <f t="shared" si="6"/>
-        <v>11.854794520547944</v>
-      </c>
-      <c r="R4" s="7">
-        <f t="shared" si="7"/>
-        <v>8.3050847457627114E-2</v>
-      </c>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="7"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -922,22 +870,10 @@
         <f t="shared" si="3"/>
         <v>0.10508474576271186</v>
       </c>
-      <c r="O5" s="6">
-        <f t="shared" si="4"/>
-        <v>12.619718309859154</v>
-      </c>
-      <c r="P5" s="6">
-        <f t="shared" si="5"/>
-        <v>1.0877118644067796</v>
-      </c>
-      <c r="Q5" s="6">
-        <f t="shared" si="6"/>
-        <v>10.350806451612904</v>
-      </c>
-      <c r="R5" s="7">
-        <f t="shared" si="7"/>
-        <v>6.0169491525423731E-2</v>
-      </c>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="7"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -986,22 +922,10 @@
         <f t="shared" si="3"/>
         <v>0.28474576271186441</v>
       </c>
-      <c r="O6" s="6">
-        <f t="shared" si="4"/>
-        <v>20.329439252336449</v>
-      </c>
-      <c r="P6" s="6">
-        <f t="shared" si="5"/>
-        <v>4.0152542372881355</v>
-      </c>
-      <c r="Q6" s="6">
-        <f t="shared" si="6"/>
-        <v>14.101190476190476</v>
-      </c>
-      <c r="R6" s="7">
-        <f t="shared" si="7"/>
-        <v>0.18135593220338983</v>
-      </c>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="7"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1050,22 +974,10 @@
         <f t="shared" si="3"/>
         <v>7.7118644067796616E-2</v>
       </c>
-      <c r="O7" s="6">
-        <f t="shared" si="4"/>
-        <v>12.742718446601941</v>
-      </c>
-      <c r="P7" s="6">
-        <f t="shared" si="5"/>
-        <v>0.88453389830508478</v>
-      </c>
-      <c r="Q7" s="6">
-        <f t="shared" si="6"/>
-        <v>11.469780219780219</v>
-      </c>
-      <c r="R7" s="7">
-        <f t="shared" si="7"/>
-        <v>4.3644067796610168E-2</v>
-      </c>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="7"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -1114,22 +1026,10 @@
         <f t="shared" si="3"/>
         <v>0.13389830508474576</v>
       </c>
-      <c r="O8" s="6">
-        <f t="shared" si="4"/>
-        <v>20.081395348837209</v>
-      </c>
-      <c r="P8" s="6">
-        <f t="shared" si="5"/>
-        <v>1.791949152542373</v>
-      </c>
-      <c r="Q8" s="6">
-        <f t="shared" si="6"/>
-        <v>13.382911392405063</v>
-      </c>
-      <c r="R8" s="7">
-        <f t="shared" si="7"/>
-        <v>7.2881355932203393E-2</v>
-      </c>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="7"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -1178,22 +1078,10 @@
         <f t="shared" si="3"/>
         <v>0.2135593220338983</v>
       </c>
-      <c r="O9" s="6">
-        <f t="shared" si="4"/>
-        <v>15.845945945945946</v>
-      </c>
-      <c r="P9" s="6">
-        <f t="shared" si="5"/>
-        <v>2.3158474576271186</v>
-      </c>
-      <c r="Q9" s="6">
-        <f t="shared" si="6"/>
-        <v>10.844047619047618</v>
-      </c>
-      <c r="R9" s="7">
-        <f t="shared" si="7"/>
-        <v>0.12542372881355932</v>
-      </c>
+      <c r="O9" s="6"/>
+      <c r="P9" s="6"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="7"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -1242,22 +1130,10 @@
         <f t="shared" si="3"/>
         <v>0.31567796610169491</v>
       </c>
-      <c r="O10" s="6">
-        <f t="shared" si="4"/>
-        <v>27.44813278008299</v>
-      </c>
-      <c r="P10" s="6">
-        <f t="shared" si="5"/>
-        <v>5.9343220338983054</v>
-      </c>
-      <c r="Q10" s="6">
-        <f t="shared" si="6"/>
-        <v>18.798657718120804</v>
-      </c>
-      <c r="R10" s="7">
-        <f t="shared" si="7"/>
-        <v>0.20423728813559322</v>
-      </c>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="7"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
@@ -1306,22 +1182,10 @@
         <f t="shared" si="3"/>
         <v>6.5677966101694921E-2</v>
       </c>
-      <c r="O11" s="6">
-        <f t="shared" si="4"/>
-        <v>12.071428571428571</v>
-      </c>
-      <c r="P11" s="6">
-        <f t="shared" si="5"/>
-        <v>0.75805084745762707</v>
-      </c>
-      <c r="Q11" s="6">
-        <f t="shared" si="6"/>
-        <v>11.541935483870967</v>
-      </c>
-      <c r="R11" s="7">
-        <f t="shared" si="7"/>
-        <v>3.5593220338983052E-2</v>
-      </c>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="7"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -1370,22 +1234,10 @@
         <f t="shared" si="3"/>
         <v>0.14745762711864407</v>
       </c>
-      <c r="O12" s="6">
-        <f t="shared" si="4"/>
-        <v>18.621105527638193</v>
-      </c>
-      <c r="P12" s="6">
-        <f t="shared" si="5"/>
-        <v>1.8985593220338983</v>
-      </c>
-      <c r="Q12" s="6">
-        <f t="shared" si="6"/>
-        <v>12.87528735632184</v>
-      </c>
-      <c r="R12" s="7">
-        <f t="shared" si="7"/>
-        <v>8.4322033898305088E-2</v>
-      </c>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="7"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -1434,22 +1286,10 @@
         <f t="shared" si="3"/>
         <v>0.19491525423728814</v>
       </c>
-      <c r="O13" s="6">
-        <f t="shared" si="4"/>
-        <v>19.540659340659342</v>
-      </c>
-      <c r="P13" s="6">
-        <f t="shared" si="5"/>
-        <v>2.5888135593220341</v>
-      </c>
-      <c r="Q13" s="6">
-        <f t="shared" si="6"/>
-        <v>13.281739130434783</v>
-      </c>
-      <c r="R13" s="7">
-        <f t="shared" si="7"/>
-        <v>0.11567796610169491</v>
-      </c>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="7"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
@@ -1498,22 +1338,10 @@
         <f t="shared" si="3"/>
         <v>8.5593220338983048E-2</v>
       </c>
-      <c r="O14" s="6">
-        <f t="shared" si="4"/>
-        <v>18.078260869565216</v>
-      </c>
-      <c r="P14" s="6">
-        <f t="shared" si="5"/>
-        <v>1.2093220338983051</v>
-      </c>
-      <c r="Q14" s="6">
-        <f t="shared" si="6"/>
-        <v>14.128712871287128</v>
-      </c>
-      <c r="R14" s="7">
-        <f t="shared" si="7"/>
-        <v>4.8728813559322036E-2</v>
-      </c>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="7"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
@@ -1562,22 +1390,10 @@
         <f t="shared" si="3"/>
         <v>0.11779661016949153</v>
       </c>
-      <c r="O15" s="6">
-        <f t="shared" si="4"/>
-        <v>19.485714285714288</v>
-      </c>
-      <c r="P15" s="6">
-        <f t="shared" si="5"/>
-        <v>1.6577118644067796</v>
-      </c>
-      <c r="Q15" s="6">
-        <f t="shared" si="6"/>
-        <v>14.072661870503596</v>
-      </c>
-      <c r="R15" s="7">
-        <f t="shared" si="7"/>
-        <v>6.8220338983050841E-2</v>
-      </c>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="7"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -1626,22 +1442,10 @@
         <f t="shared" si="3"/>
         <v>0.17542372881355933</v>
       </c>
-      <c r="O16" s="6">
-        <f t="shared" si="4"/>
-        <v>18.695358649789029</v>
-      </c>
-      <c r="P16" s="6">
-        <f t="shared" si="5"/>
-        <v>2.2058474576271188</v>
-      </c>
-      <c r="Q16" s="6">
-        <f t="shared" si="6"/>
-        <v>12.574396135265701</v>
-      </c>
-      <c r="R16" s="7">
-        <f t="shared" si="7"/>
-        <v>0.10042372881355932</v>
-      </c>
+      <c r="O16" s="6"/>
+      <c r="P16" s="6"/>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>